<commit_message>
data: update records 2026-10-06
</commit_message>
<xml_diff>
--- a/public/records.xlsx
+++ b/public/records.xlsx
@@ -3691,27 +3691,27 @@
       <c r="E67" t="inlineStr"/>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>21.73</t>
+          <t>21.64</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>21.73</t>
+          <t>21.64</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>Казань</t>
+          <t>Баку</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>07.11.2025</t>
+          <t>03.10.2026</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>2025-11-07</t>
+          <t>2026-10-03</t>
         </is>
       </c>
     </row>
@@ -3733,33 +3733,33 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Морозов Владимир</t>
+          <t>Корнев Егор</t>
         </is>
       </c>
       <c r="E68" t="inlineStr"/>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>20.31</t>
+          <t>20.26</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>20.31</t>
+          <t>20.26</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>Копенгаген</t>
+          <t>Баку</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>15.12.2017</t>
+          <t>01.10.2026</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>2017-12-15</t>
+          <t>2026-10-01</t>
         </is>
       </c>
     </row>
@@ -3925,33 +3925,33 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Морозов Владимир</t>
+          <t>Корнев Егор</t>
         </is>
       </c>
       <c r="E72" t="inlineStr"/>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>44.95</t>
+          <t>44.84</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>44.95</t>
+          <t>44.84</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>Сингапур</t>
+          <t>Баку</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>16.11.2018</t>
+          <t>02.10.2026</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>2018-11-16</t>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
@@ -6997,17 +6997,17 @@
       <c r="C4" t="inlineStr"/>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>21.73</t>
+          <t>21.64</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Казань</t>
+          <t>Баку</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>07.11.2025</t>
+          <t>03.10.2026</t>
         </is>
       </c>
     </row>
@@ -7019,23 +7019,23 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Морозов Владимир</t>
+          <t>Корнев Егор</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>20.31</t>
+          <t>20.26</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Копенгаген</t>
+          <t>Баку</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>15.12.2017</t>
+          <t>01.10.2026</t>
         </is>
       </c>
     </row>
@@ -7131,23 +7131,23 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Морозов Владимир</t>
+          <t>Корнев Егор</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>44.95</t>
+          <t>44.84</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Сингапур</t>
+          <t>Баку</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>16.11.2018</t>
+          <t>02.10.2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: update records 2026-10-11
</commit_message>
<xml_diff>
--- a/public/records.xlsx
+++ b/public/records.xlsx
@@ -3691,27 +3691,27 @@
       <c r="E67" t="inlineStr"/>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>21.64</t>
+          <t>21.28</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>21.64</t>
+          <t>21.28</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>Баку</t>
+          <t>Ташкент</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>03.10.2026</t>
+          <t>10.10.2026</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-10</t>
         </is>
       </c>
     </row>
@@ -6997,17 +6997,17 @@
       <c r="C4" t="inlineStr"/>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>21.64</t>
+          <t>21.28</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Баку</t>
+          <t>Ташкент</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>03.10.2026</t>
+          <t>10.10.2026</t>
         </is>
       </c>
     </row>

</xml_diff>